<commit_message>
chore: make state_model=WAIVER explicit in the example basis
examples/data/basis.xlsx relied on the implicit `waiver_table` -> `WAIVER_MODEL`
fallback; declare `state_model=WAIVER` on the segments defaults row, matching the
bundled sample. Behaviour-neutral -- the same WAIVER state model was already
applied (543 tests pass).
</commit_message>
<xml_diff>
--- a/examples/data/basis.xlsx
+++ b/examples/data/basis.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,11 @@
           <t>surrender_value_table</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>state_model</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -594,6 +599,11 @@
       <c r="S2" t="inlineStr">
         <is>
           <t>SURRENDER_STD</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>WAIVER</t>
         </is>
       </c>
     </row>

</xml_diff>